<commit_message>
fix(brand): coming-soon page uses the zomo logo and lowercase name
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/translation/georgian-translation.xlsx
+++ b/translation/georgian-translation.xlsx
@@ -42657,12 +42657,12 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>We're getting Zomo ready for launch. See you soon.</t>
+          <t>We're getting zomo ready for launch. See you soon.</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Zomo-ს გასაშვებად ვამზადებთ. მალე შევხვდებით.</t>
+          <t>ზომოს გასაშვებად ვამზადებთ. მალე შევხვდებით.</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -42723,12 +42723,12 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Zomo — Coming soon</t>
+          <t>zomo — Coming soon</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Zomo — მალე</t>
+          <t>ზომო — მალე</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">

</xml_diff>